<commit_message>
fix(varredura): recuperacao robusta, semanas dinamicas e atualizacao ate 22/09 com loja 19891 consolidada
</commit_message>
<xml_diff>
--- a/dados_all_stores/Keys Summary - All Stores (Stores) (2026-09-07).xlsx
+++ b/dados_all_stores/Keys Summary - All Stores (Stores) (2026-09-07).xlsx
@@ -912,33 +912,33 @@
   </si>
   <si>
     <t>214
-174</t>
-  </si>
-  <si>
-    <t>24</t>
-  </si>
-  <si>
-    <t>R$ 1.591.647,88</t>
-  </si>
-  <si>
-    <t>R$ 8.421,42
-R$ 8.543,05</t>
-  </si>
-  <si>
-    <t>157.6%
-160.7%</t>
-  </si>
-  <si>
-    <t>92.2</t>
-  </si>
-  <si>
-    <t>131.0%</t>
-  </si>
-  <si>
-    <t>52.7%</t>
-  </si>
-  <si>
-    <t>10.7%</t>
+175</t>
+  </si>
+  <si>
+    <t>23</t>
+  </si>
+  <si>
+    <t>R$ 1.597.733,91</t>
+  </si>
+  <si>
+    <t>R$ 8.409,13
+R$ 8.529,01</t>
+  </si>
+  <si>
+    <t>157.5%
+160.6%</t>
+  </si>
+  <si>
+    <t>92.1</t>
+  </si>
+  <si>
+    <t>130.9%</t>
+  </si>
+  <si>
+    <t>52.5%</t>
+  </si>
+  <si>
+    <t>10.5%</t>
   </si>
   <si>
     <t>2.3%</t>
@@ -947,34 +947,34 @@
     <t>0.2%</t>
   </si>
   <si>
-    <t>35.4</t>
-  </si>
-  <si>
-    <t>47.8%</t>
-  </si>
-  <si>
-    <t>27.8%</t>
+    <t>35.7</t>
+  </si>
+  <si>
+    <t>47.7%</t>
+  </si>
+  <si>
+    <t>28.0%</t>
   </si>
   <si>
     <t>8.8</t>
   </si>
   <si>
-    <t>10.8</t>
+    <t>11.0</t>
   </si>
   <si>
     <t>20.3</t>
   </si>
   <si>
-    <t>26.1</t>
-  </si>
-  <si>
-    <t>49.3%</t>
-  </si>
-  <si>
-    <t>-R$ 46.909,60</t>
-  </si>
-  <si>
-    <t>2.97</t>
+    <t>26.4</t>
+  </si>
+  <si>
+    <t>49.2%</t>
+  </si>
+  <si>
+    <t>-R$ 46.987,60</t>
+  </si>
+  <si>
+    <t>2.94</t>
   </si>
   <si>
     <t>3.52</t>
@@ -10137,7 +10137,7 @@
         <v>19647</v>
       </c>
       <c r="B69" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="s" r="C69" s="4">
         <v>44</v>
@@ -10171,27 +10171,61 @@
       <c t="s" r="N69" s="4">
         <v>52</v>
       </c>
-      <c r="O69" s="5"/>
-      <c r="P69" s="5"/>
-      <c r="Q69" s="6"/>
-      <c r="R69" s="7"/>
-      <c r="S69" s="6"/>
-      <c r="T69" s="6"/>
-      <c r="U69" s="6"/>
-      <c r="V69" s="6"/>
-      <c r="W69" s="6"/>
-      <c r="X69" s="8"/>
-      <c r="Y69" s="6"/>
-      <c r="Z69" s="6"/>
-      <c r="AA69" s="8"/>
-      <c r="AB69" s="8"/>
+      <c r="O69" s="5">
+        <v>6086.0299999999997</v>
+      </c>
+      <c r="P69" s="5">
+        <v>6086.0299999999997</v>
+      </c>
+      <c r="Q69" s="6">
+        <v>1.4482199605776578</v>
+      </c>
+      <c r="R69" s="7">
+        <v>67</v>
+      </c>
+      <c r="S69" s="6">
+        <v>1.161290322580645</v>
+      </c>
+      <c r="T69" s="6">
+        <v>-0.13049327722669787</v>
+      </c>
+      <c r="U69" s="6">
+        <v>-0.4297425415254279</v>
+      </c>
+      <c r="V69" s="6">
+        <v>0.020369436233472395</v>
+      </c>
+      <c r="W69" s="6">
+        <v>-0.011539706508183496</v>
+      </c>
+      <c r="X69" s="8">
+        <v>96.96632653061225</v>
+      </c>
+      <c r="Y69" s="6">
+        <v>0.22448979591836735</v>
+      </c>
+      <c r="Z69" s="6">
+        <v>0.77551020408163263</v>
+      </c>
+      <c r="AA69" s="8">
+        <v>7.4921573529411765</v>
+      </c>
+      <c r="AB69" s="8">
+        <v>63.632312244897953</v>
+      </c>
       <c r="AC69" s="8">
         <v>71.525121999999996</v>
       </c>
-      <c r="AD69" s="8"/>
-      <c r="AE69" s="6"/>
+      <c r="AD69" s="8">
+        <v>79.394218367346937</v>
+      </c>
+      <c r="AE69" s="6">
+        <v>0.12244897959183673</v>
+      </c>
       <c r="AF69" s="9"/>
-      <c r="AG69" s="5"/>
+      <c r="AG69" s="5">
+        <v>-78</v>
+      </c>
       <c r="AH69" s="10">
         <v>2</v>
       </c>
@@ -11031,7 +11065,7 @@
         <v>0.016253450011701996</v>
       </c>
       <c r="W76" s="6">
-        <v>-0.012030760325107775</v>
+        <v>-0.013851840260130536</v>
       </c>
       <c r="X76" s="8">
         <v>31.238775510204082</v>
@@ -15437,7 +15471,7 @@
         <v>0</v>
       </c>
       <c r="AH111" s="10">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AI111" s="11"/>
       <c r="AJ111" s="13">
@@ -15782,7 +15816,7 @@
         <v>0</v>
       </c>
       <c r="AH114" s="10">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AI114" s="11"/>
       <c r="AJ114" s="13">
@@ -17312,7 +17346,7 @@
         <v>0</v>
       </c>
       <c r="AH126" s="10">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AI126" s="11"/>
       <c r="AJ126" s="13">
@@ -18489,7 +18523,7 @@
         <v>0</v>
       </c>
       <c r="AH135" s="10">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AI135" s="11"/>
       <c r="AJ135" s="13">
@@ -20807,7 +20841,7 @@
         <v>-2534.6500000000001</v>
       </c>
       <c r="AH153" s="10">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AI153" s="11"/>
       <c r="AJ153" s="13">
@@ -22091,7 +22125,7 @@
         <v>-1484.04</v>
       </c>
       <c r="AH163" s="10">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AI163" s="11"/>
       <c r="AJ163" s="13">
@@ -28254,7 +28288,7 @@
       <c r="AF212" s="9"/>
       <c r="AG212" s="5"/>
       <c r="AH212" s="10">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AI212" s="11"/>
       <c r="AJ212" s="12"/>

</xml_diff>